<commit_message>
Conceptformulier Bijlage 2 bijgewerkt naar calculatiemodel v3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DGWo8ViGGiHX3nPEze7SXS
</commit_message>
<xml_diff>
--- a/calculatie/CONCEPT_Bijlage_2_Inschrijfstaat_Thebe22_VDL.xlsx
+++ b/calculatie/CONCEPT_Bijlage_2_Inschrijfstaat_Thebe22_VDL.xlsx
@@ -1424,7 +1424,7 @@
       </c>
       <c r="D14" s="12" t="n"/>
       <c r="E14" s="47" t="n">
-        <v>89750</v>
+        <v>98250</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D15" s="12" t="n"/>
       <c r="E15" s="47" t="n">
-        <v>199570</v>
+        <v>208410</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="D24" s="12" t="n"/>
       <c r="E24" s="47" t="n">
-        <v>94225</v>
+        <v>95025</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D25" s="12" t="n"/>
       <c r="E25" s="47" t="n">
-        <v>256820</v>
+        <v>262120</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="D27" s="12" t="n"/>
       <c r="E27" s="47" t="n">
-        <v>15750</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="D29" s="12" t="n"/>
       <c r="E29" s="47" t="n">
-        <v>37645</v>
+        <v>27525</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="D32" s="12" t="n"/>
       <c r="E32" s="47" t="n">
-        <v>13000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="E38" s="47" t="n">
-        <v>68700</v>
+        <v>64600</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -1726,7 +1726,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E39" s="47" t="n">
-        <v>90898</v>
+        <v>90791</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -1740,7 +1740,7 @@
         <v>0.03</v>
       </c>
       <c r="E40" s="47" t="n">
-        <v>41683</v>
+        <v>41634</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
@@ -1754,7 +1754,7 @@
         <v>0.0025</v>
       </c>
       <c r="E41" s="47" t="n">
-        <v>3578</v>
+        <v>3574</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Calculatiemodel v4: bouwkundige bijlagen 1 t/m 4 verwerkt
Vloeroppervlakken gemeten op Bijlage 3, brandscheidingen (30/60 min) op
Bijlage 4, folie op hergebruikte glazen puien, EI60-deuren, aluminium
balustrade. Nieuwe risico's: werk op 1e/2e verdieping en terreininrichting
uit Bijlage 1, en twee afwijkende versies van de plattegrond.
Conceptformulier bijgewerkt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DGWo8ViGGiHX3nPEze7SXS
</commit_message>
<xml_diff>
--- a/calculatie/CONCEPT_Bijlage_2_Inschrijfstaat_Thebe22_VDL.xlsx
+++ b/calculatie/CONCEPT_Bijlage_2_Inschrijfstaat_Thebe22_VDL.xlsx
@@ -1545,7 +1545,7 @@
       </c>
       <c r="D24" s="12" t="n"/>
       <c r="E24" s="47" t="n">
-        <v>95025</v>
+        <v>94673</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D25" s="12" t="n"/>
       <c r="E25" s="47" t="n">
-        <v>262120</v>
+        <v>291270</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="D30" s="12" t="n"/>
       <c r="E30" s="47" t="n">
-        <v>6750</v>
+        <v>8550</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="E34" s="47" t="n">
-        <v>8500</v>
+        <v>23200</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -1726,7 +1726,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E39" s="47" t="n">
-        <v>90791</v>
+        <v>93962</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -1740,7 +1740,7 @@
         <v>0.03</v>
       </c>
       <c r="E40" s="47" t="n">
-        <v>41634</v>
+        <v>43088</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
@@ -1754,7 +1754,7 @@
         <v>0.0025</v>
       </c>
       <c r="E41" s="47" t="n">
-        <v>3574</v>
+        <v>3698</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Calculatiemodel v5: offerte Trigion, afzuigkappen en toegangscontrole verwerkt
Bekabeling toegangscontrole (29 deuren naar centrale controllers) en
camera's, 230V-punten voor Trigion-apparatuur, afzuigkappen op basis van
offerte Techno Horeca OV260801 + montage. Nieuwe risico's: coördinatie
Trigion, deurcontacten, capaciteit plasmafilters. Conceptformulier
bijgewerkt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DGWo8ViGGiHX3nPEze7SXS
</commit_message>
<xml_diff>
--- a/calculatie/CONCEPT_Bijlage_2_Inschrijfstaat_Thebe22_VDL.xlsx
+++ b/calculatie/CONCEPT_Bijlage_2_Inschrijfstaat_Thebe22_VDL.xlsx
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D15" s="12" t="n"/>
       <c r="E15" s="47" t="n">
-        <v>208410</v>
+        <v>189403</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="D17" s="12" t="n"/>
       <c r="E17" s="47" t="n">
-        <v>54680</v>
+        <v>56240</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="D19" s="12" t="n"/>
       <c r="E19" s="47" t="n">
-        <v>12700</v>
+        <v>26630</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="D36" s="12" t="n"/>
       <c r="E36" s="47" t="n">
-        <v>49000</v>
+        <v>50200</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -1726,7 +1726,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E39" s="47" t="n">
-        <v>93962</v>
+        <v>93800</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -1740,7 +1740,7 @@
         <v>0.03</v>
       </c>
       <c r="E40" s="47" t="n">
-        <v>43088</v>
+        <v>43014</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
@@ -1754,7 +1754,7 @@
         <v>0.0025</v>
       </c>
       <c r="E41" s="47" t="n">
-        <v>3698</v>
+        <v>3692</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">

</xml_diff>